<commit_message>
def fix for older phase 2 evals
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/AggregateResults/Variable Definitions/PH2_Variables.xlsx
+++ b/dashboard-ui/src/components/AggregateResults/Variable Definitions/PH2_Variables.xlsx
@@ -46,22 +46,22 @@
     <t>Trust</t>
   </si>
   <si>
-    <t>AF_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>MF_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>PS_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>SS_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>PS_Multi_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>AF_Multi_KDMA_TEXT</t>
+    <t>AF_KDMA_Text</t>
+  </si>
+  <si>
+    <t>MF_KDMA_Text</t>
+  </si>
+  <si>
+    <t>PS_KDMA_Text</t>
+  </si>
+  <si>
+    <t>SS_KDMA_Text</t>
+  </si>
+  <si>
+    <t>PS_Multi_KDMA_Text</t>
+  </si>
+  <si>
+    <t>AF_Multi_KDMA_Text</t>
   </si>
   <si>
     <t>Variable Group</t>
@@ -548,8 +548,8 @@
     <col min="11" max="11" style="2" width="73.005" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="2" width="73.005" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="2" width="73.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="2" width="57.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="2" width="84.14785714285713" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="2" width="73.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Itm 1391: June 2026 Participant-level (#491)
* it works

* replace some bad code

* vars

* load it

* more refactoring

* def fix for older phase 2 evals
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/AggregateResults/Variable Definitions/PH2_Variables.xlsx
+++ b/dashboard-ui/src/components/AggregateResults/Variable Definitions/PH2_Variables.xlsx
@@ -19,7 +19,7 @@
     <t>Variable</t>
   </si>
   <si>
-    <t>ParticipantID</t>
+    <t>Participant ID</t>
   </si>
   <si>
     <t>Date</t>
@@ -46,22 +46,22 @@
     <t>Trust</t>
   </si>
   <si>
-    <t>AF_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>MF_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>PS_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>SS_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>PS_Multi_KDMA_TEXT</t>
-  </si>
-  <si>
-    <t>AF_Multi_KDMA_TEXT</t>
+    <t>AF_KDMA_Text</t>
+  </si>
+  <si>
+    <t>MF_KDMA_Text</t>
+  </si>
+  <si>
+    <t>PS_KDMA_Text</t>
+  </si>
+  <si>
+    <t>SS_KDMA_Text</t>
+  </si>
+  <si>
+    <t>PS_Multi_KDMA_Text</t>
+  </si>
+  <si>
+    <t>AF_Multi_KDMA_Text</t>
   </si>
   <si>
     <t>Variable Group</t>
@@ -222,16 +222,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -551,8 +548,8 @@
     <col min="11" max="11" style="2" width="73.005" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="2" width="73.005" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="2" width="73.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="3" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="3" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="2" width="57.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="2" width="84.14785714285713" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="2" width="73.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>

</xml_diff>